<commit_message>
Bug fixes, and additionally features added in features insert script.
</commit_message>
<xml_diff>
--- a/docs_repo/notes.xlsx
+++ b/docs_repo/notes.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\DESKTOP\ERP\docs_repo\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="11_F25DC773A252ABDACC104816B1D97C865BDE58EF" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FE6CF666-26BF-4A3B-8175-782F24C2F8E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="32340" yWindow="1260" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -24,11 +24,396 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="27" uniqueCount="27">
+  <si>
+    <r>
+      <t xml:space="preserve">You already have the two </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>incoming</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> screens. What you need next are the screens for </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>outgoing, movement, control, and visibility</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>. A usable inventory module usually includes receipts, deliveries, transfers, adjustments, reservations, and stock views.frappe+2</t>
+    </r>
+  </si>
+  <si>
+    <t>Must-have next screens</t>
+  </si>
+  <si>
+    <r>
+      <t>Delivery / Goods Issue</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, stock out against sales order or manual issue.tenthplanet+1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Stock Transfer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, warehouse-to-warehouse movement.pantrysoft+1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Stock Adjustment</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, increase/decrease for damage, count difference, scrap, opening balance correction.oracle+1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Stock Reservation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, reserve stock against sales orders.alcaidc+1</t>
+    </r>
+  </si>
+  <si>
+    <t>Visibility screens</t>
+  </si>
+  <si>
+    <r>
+      <t>Inventory Summary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, current on-hand, reserved, available, in-transit by material and warehouse.pattern+1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Stock Ledger</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, full movement history for every IN/OUT transaction.quickdiceerp+1</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Low Stock / Reorder</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, show items below reorder level.deskera+1</t>
+    </r>
+  </si>
+  <si>
+    <t>Useful operational screens</t>
+  </si>
+  <si>
+    <r>
+      <t>Material-wise stock view</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Warehouse-wise stock view</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Pending receipts / pending deliveries</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>Transfer status screen</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, draft, in transit, received.veeqo+2</t>
+    </r>
+  </si>
+  <si>
+    <t>Best next build order</t>
+  </si>
+  <si>
+    <r>
+      <t>1. Delivery / Goods Issue</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>2. Stock Reservation</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>3. Stock Transfer</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>4. Stock Adjustment</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>5. Inventory Summary</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t>6. Stock Ledger report</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.alcaidc+2</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">For your current setup, the </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>very next screens</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> should be:</t>
+    </r>
+  </si>
+  <si>
+    <t>Delivery</t>
+  </si>
+  <si>
+    <t>Stock Transfer</t>
+  </si>
+  <si>
+    <t>Stock Adjustment</t>
+  </si>
+  <si>
+    <r>
+      <t>Inventory Summary / Stock Ledger</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>frappe+2</t>
+    </r>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="18"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
@@ -55,8 +440,23 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="2"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -337,9 +737,244 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1"/>
+  <dimension ref="A1:A65"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <sheetData>
+    <row r="1" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="3" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="4" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A4" s="2"/>
+    </row>
+    <row r="5" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A5" s="3" t="s">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="6" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A6" s="2"/>
+    </row>
+    <row r="7" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A7" s="3" t="s">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A8" s="2"/>
+    </row>
+    <row r="9" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A9" s="3" t="s">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="10" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A10" s="2"/>
+    </row>
+    <row r="11" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A11" s="3" t="s">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="14" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A14" s="2"/>
+    </row>
+    <row r="15" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A15" s="3" t="s">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A16" s="2"/>
+    </row>
+    <row r="17" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A17" s="3" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A18" s="2"/>
+    </row>
+    <row r="19" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A19" s="3" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="21" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A21" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="22" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A22" s="2"/>
+    </row>
+    <row r="23" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A23" s="3" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="24" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A24" s="2"/>
+    </row>
+    <row r="25" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A25" s="3" t="s">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="26" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A26" s="2"/>
+    </row>
+    <row r="27" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A27" s="3" t="s">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="28" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A28" s="2"/>
+    </row>
+    <row r="29" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A29" s="3" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="31" spans="1:1" ht="23.25" x14ac:dyDescent="0.25">
+      <c r="A31" s="1" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="32" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A32" s="2"/>
+    </row>
+    <row r="33" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A33" s="2"/>
+    </row>
+    <row r="34" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A34" s="4"/>
+    </row>
+    <row r="35" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A35" s="5" t="s">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="36" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A36" s="2"/>
+    </row>
+    <row r="37" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A37" s="2"/>
+    </row>
+    <row r="38" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A38" s="4"/>
+    </row>
+    <row r="39" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A39" s="5" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="40" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A40" s="2"/>
+    </row>
+    <row r="41" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A41" s="2"/>
+    </row>
+    <row r="42" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A42" s="4"/>
+    </row>
+    <row r="43" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A43" s="5" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="44" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A44" s="2"/>
+    </row>
+    <row r="45" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A45" s="2"/>
+    </row>
+    <row r="46" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A46" s="4"/>
+    </row>
+    <row r="47" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A47" s="5" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="48" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A48" s="2"/>
+    </row>
+    <row r="49" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A49" s="2"/>
+    </row>
+    <row r="50" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A50" s="4"/>
+    </row>
+    <row r="51" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A51" s="5" t="s">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="52" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A52" s="2"/>
+    </row>
+    <row r="53" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A53" s="2"/>
+    </row>
+    <row r="54" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A54" s="4"/>
+    </row>
+    <row r="55" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A55" s="5" t="s">
+        <v>21</v>
+      </c>
+    </row>
+    <row r="57" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A57" t="s">
+        <v>22</v>
+      </c>
+    </row>
+    <row r="58" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A58" s="2"/>
+    </row>
+    <row r="59" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A59" s="3" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="60" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A60" s="2"/>
+    </row>
+    <row r="61" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A61" s="3" t="s">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="62" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A62" s="2"/>
+    </row>
+    <row r="63" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A63" s="3" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="64" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A64" s="2"/>
+    </row>
+    <row r="65" spans="1:1" x14ac:dyDescent="0.25">
+      <c r="A65" s="3" t="s">
+        <v>26</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>